<commit_message>
Add Sika Automotive reports and update audit for all 12 customers
- build_sika_atm_de_report.py: KNR 413276+493163 combined (20 Cluster, -1,603 EUR)
- build_sika_527406_report.py: KNR 527406 (21 Cluster, -13,994 EUR)
- build_audit_report.py: extended to 12 customers incl. both Sika Automotive entities
- 00_audit_extraktion.xlsx regenerated with all customers

https://claude.ai/code/session_01QY1f1VNnd5RWsUcy3L3Squ
</commit_message>
<xml_diff>
--- a/output/billing_report/00_audit_extraktion.xlsx
+++ b/output/billing_report/00_audit_extraktion.xlsx
@@ -18,6 +18,8 @@
     <sheet name="EBM-Papst Mulfingen" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Fischerwerke GmbH &amp; Co KG" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Groz-Beckert KG" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Sika Automotive AG" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Sika Automotive DE" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -516,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH12"/>
+  <dimension ref="A1:AH14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1854,6 +1856,226 @@
         <v>0</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Sika Automotive AG</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>527406</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>303</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>420</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="M13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="N13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="O13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="5" t="n">
+        <v>96</v>
+      </c>
+      <c r="Q13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="R13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="S13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="T13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="U13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="V13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="W13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="X13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="Y13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="Z13" s="5" t="n">
+        <v>98.3</v>
+      </c>
+      <c r="AA13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AC13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AD13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AE13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AF13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AH13" s="5" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Sika Automotive DE</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>413276+493163</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>448</v>
+      </c>
+      <c r="I14" s="8" t="n">
+        <v>481</v>
+      </c>
+      <c r="J14" s="8" t="n">
+        <v>64</v>
+      </c>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="M14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="N14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="O14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="R14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="S14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="T14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="U14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="V14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="W14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="X14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="Y14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="Z14" s="5" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="AA14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AC14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AD14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AE14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AF14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AH14" s="5" t="n">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:AH1"/>
@@ -3428,6 +3650,1572 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Daten-Qualität: Sika Automotive AG</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>Quelle</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>Feld</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>N Zeilen</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>Gefüllt%</t>
+        </is>
+      </c>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>Fehlt%</t>
+        </is>
+      </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
+          <t>Bewertung</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>bi_raw</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Empfänger Land</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>303</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>bi_raw</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Empfänger PLZ</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>303</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>bi_raw</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Tonnage (eff.)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>303</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>bi_raw</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Stellplätze</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>303</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>✗ Lückenhaft</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>bi_raw</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Lademeter</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>303</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>96</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>bi_raw</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Volumen</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>303</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>bi_raw</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Leistungsdatum</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>303</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Dinas Fracht</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>303</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Dinas Diesel</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>303</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Dinas Maut/SSD</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>303</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Dinas Gesamt</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>303</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Empfänger Land</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>420</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Empfänger PLZ</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>420</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Tonnage (eff.)</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>420</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Stellplätze</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>420</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>98.3</v>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Lademeter</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>420</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Volumen</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>420</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Leistungsdatum</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>420</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F20" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>AX Fracht</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>420</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>AX Diesel</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>420</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F22" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>AX Maut</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>420</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>AX Nebengebühr</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>420</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F24" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>AX Gesamt</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>420</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Daten-Qualität: Sika Automotive DE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>Quelle</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>Feld</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>N Zeilen</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>Gefüllt%</t>
+        </is>
+      </c>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>Fehlt%</t>
+        </is>
+      </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
+          <t>Bewertung</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>bi_raw</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Empfänger Land</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>448</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>bi_raw</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Empfänger PLZ</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>448</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>bi_raw</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Tonnage (eff.)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>448</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>bi_raw</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Stellplätze</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>448</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>✗ Lückenhaft</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>bi_raw</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Lademeter</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>448</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>bi_raw</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Volumen</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>448</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>bi_raw</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Leistungsdatum</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>448</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Dinas Fracht</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>448</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Dinas Diesel</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>448</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Dinas Maut/SSD</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>448</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Dinas Gesamt</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>448</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Empfänger Land</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>481</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Empfänger PLZ</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>481</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Tonnage (eff.)</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>481</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Stellplätze</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>481</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Lademeter</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>481</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Volumen</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>481</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Leistungsdatum</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>481</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F20" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>AX Fracht</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>481</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>AX Diesel</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>481</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F22" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>AX Maut</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>481</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>AX Nebengebühr</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>481</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F24" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>AX/BI</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>AX Gesamt</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>481</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>✓ OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Fix audit data problems: HERMA paths, Groz-Beckert POST from BI, metric rename
- HERMA: correct DINAS/AX PDF paths to data/extracted/bi/Herma/...
- Groz-Beckert: load POST from full BI (KNRs 410912/490527/527410/527373) → 754 POST rows
- Rename 'DINAS fehlgeschlagen' → 'DINAS 0-Pos/Cover PDFs' (Fischer issue clarified)
- Groz-Beckert KNR set to 410912

https://claude.ai/code/session_01QY1f1VNnd5RWsUcy3L3Squ
</commit_message>
<xml_diff>
--- a/output/billing_report/00_audit_extraktion.xlsx
+++ b/output/billing_report/00_audit_extraktion.xlsx
@@ -597,7 +597,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>DINAS fehlgeschlagen (ca.)</t>
+          <t>DINAS 0-Pos/Cover PDFs</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -1084,10 +1084,10 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>0</v>
+        <v>319</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>0</v>
+        <v>333</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>442</v>
@@ -1096,7 +1096,7 @@
         <v>275</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="H6" s="8" t="n">
         <v>323</v>
@@ -1752,7 +1752,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>410912</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
@@ -1774,12 +1774,10 @@
         <v>1854</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="7" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
+        <v>754</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>15</v>
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
@@ -1819,41 +1817,41 @@
       <c r="V12" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="W12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="X12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH12" s="6" t="n">
-        <v>0</v>
+      <c r="W12" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="X12" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="Y12" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="Z12" s="5" t="n">
+        <v>98</v>
+      </c>
+      <c r="AA12" s="5" t="n">
+        <v>99.90000000000001</v>
+      </c>
+      <c r="AB12" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AC12" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AD12" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AE12" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AF12" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG12" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AH12" s="5" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="13">
@@ -3287,17 +3285,17 @@
         </is>
       </c>
       <c r="D14" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="6" t="n">
-        <v>0</v>
+        <v>754</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -3318,17 +3316,17 @@
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="6" t="n">
-        <v>0</v>
+        <v>754</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -3349,17 +3347,17 @@
         </is>
       </c>
       <c r="D16" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="6" t="n">
-        <v>0</v>
+        <v>754</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -3380,17 +3378,17 @@
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="6" t="n">
-        <v>0</v>
+        <v>754</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>98</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -3411,17 +3409,17 @@
         </is>
       </c>
       <c r="D18" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="6" t="n">
-        <v>0</v>
+        <v>754</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>99.90000000000001</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -3442,17 +3440,17 @@
         </is>
       </c>
       <c r="D19" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="6" t="n">
-        <v>0</v>
+        <v>754</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -3473,17 +3471,17 @@
         </is>
       </c>
       <c r="D20" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="6" t="n">
-        <v>0</v>
+        <v>754</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -3504,17 +3502,17 @@
         </is>
       </c>
       <c r="D21" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="6" t="n">
-        <v>0</v>
+        <v>754</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -3535,17 +3533,17 @@
         </is>
       </c>
       <c r="D22" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="6" t="n">
-        <v>0</v>
+        <v>754</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -3566,17 +3564,17 @@
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="6" t="n">
-        <v>0</v>
+        <v>754</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -3597,17 +3595,17 @@
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="6" t="n">
-        <v>0</v>
+        <v>754</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -3628,17 +3626,17 @@
         </is>
       </c>
       <c r="D25" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="6" t="n">
-        <v>0</v>
+        <v>754</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix HERMA completeness audit: add column rename mapping for non-standard sheet headers
HERMA's PRE/POST sheets use short names ('Land', 'PLZ', 'Tonnage kg') instead
of the standard audit field names ('Empfänger Land', 'Empfänger PLZ', 'Tonnage
(eff.)'). Added col_map parameter to CUSTOMERS config and apply rename before
pct_filled() checks. HERMA now shows 100% for all geographic and financial
fields instead of false 0%.

https://claude.ai/code/session_01QY1f1VNnd5RWsUcy3L3Squ
</commit_message>
<xml_diff>
--- a/output/billing_report/00_audit_extraktion.xlsx
+++ b/output/billing_report/00_audit_extraktion.xlsx
@@ -1091,13 +1091,13 @@
         <v>113</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>543</v>
+        <v>792</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>76</v>
+        <v>129</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>109</v>
+        <v>56</v>
       </c>
       <c r="H6" s="8" t="n">
         <v>149</v>
@@ -1203,7 +1203,7 @@
         <v>333</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>442</v>
+        <v>3298</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>275</v>
@@ -1227,20 +1227,20 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="L7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="6" t="n">
-        <v>0</v>
+      <c r="L7" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="P7" s="6" t="n">
-        <v>0</v>
+      <c r="P7" s="5" t="n">
+        <v>96.90000000000001</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>0</v>
@@ -1251,29 +1251,29 @@
       <c r="S7" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="T7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" s="6" t="n">
-        <v>0</v>
+      <c r="T7" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="U7" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="V7" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="W7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="X7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y7" s="6" t="n">
-        <v>0</v>
+      <c r="W7" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="X7" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="Y7" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="Z7" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AA7" s="6" t="n">
-        <v>0</v>
+      <c r="AA7" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="AB7" s="6" t="n">
         <v>0</v>
@@ -1284,14 +1284,14 @@
       <c r="AD7" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="AE7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG7" s="6" t="n">
-        <v>0</v>
+      <c r="AE7" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AF7" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AG7" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="AH7" s="5" t="n">
         <v>100</v>
@@ -1315,7 +1315,7 @@
         <v>2004</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>4541</v>
+        <v>4819</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>4214</v>
@@ -1427,13 +1427,13 @@
         <v>191</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>144</v>
+        <v>255</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>90</v>
+        <v>106</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="H9" s="4" t="n">
         <v>92</v>
@@ -1539,7 +1539,7 @@
         <v>155</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>382</v>
+        <v>3382</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>152</v>
@@ -1651,7 +1651,7 @@
         <v>178</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>123</v>
+        <v>613</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>118</v>
@@ -1763,13 +1763,13 @@
         <v>383</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>1347</v>
+        <v>5319</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>718</v>
+        <v>947</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>782</v>
+        <v>553</v>
       </c>
       <c r="H12" s="8" t="n">
         <v>526</v>
@@ -1903,14 +1903,14 @@
       <c r="M13" s="5" t="n">
         <v>98.90000000000001</v>
       </c>
-      <c r="N13" s="4" t="n">
-        <v>76.7</v>
+      <c r="N13" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>0</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>1</v>
+        <v>15.7</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>0</v>
@@ -3904,15 +3904,15 @@
       <c r="D5" s="4" t="n">
         <v>1854</v>
       </c>
-      <c r="E5" s="4" t="n">
-        <v>76.7</v>
+      <c r="E5" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>23.3</v>
+        <v>0</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>⚠ Teilweise</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -3967,10 +3967,10 @@
         <v>1854</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>1</v>
+        <v>15.7</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>99</v>
+        <v>84.3</v>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
@@ -9323,15 +9323,15 @@
       <c r="D3" s="4" t="n">
         <v>323</v>
       </c>
-      <c r="E3" s="6" t="n">
-        <v>0</v>
+      <c r="E3" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -9354,15 +9354,15 @@
       <c r="D4" s="4" t="n">
         <v>323</v>
       </c>
-      <c r="E4" s="6" t="n">
-        <v>0</v>
+      <c r="E4" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -9385,15 +9385,15 @@
       <c r="D5" s="4" t="n">
         <v>323</v>
       </c>
-      <c r="E5" s="6" t="n">
-        <v>0</v>
+      <c r="E5" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -9447,15 +9447,15 @@
       <c r="D7" s="4" t="n">
         <v>323</v>
       </c>
-      <c r="E7" s="6" t="n">
-        <v>0</v>
+      <c r="E7" s="5" t="n">
+        <v>96.90000000000001</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>100</v>
+        <v>3.1</v>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -9571,15 +9571,15 @@
       <c r="D11" s="4" t="n">
         <v>323</v>
       </c>
-      <c r="E11" s="6" t="n">
-        <v>0</v>
+      <c r="E11" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -9602,15 +9602,15 @@
       <c r="D12" s="4" t="n">
         <v>323</v>
       </c>
-      <c r="E12" s="6" t="n">
-        <v>0</v>
+      <c r="E12" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -9664,15 +9664,15 @@
       <c r="D14" s="8" t="n">
         <v>5112</v>
       </c>
-      <c r="E14" s="6" t="n">
-        <v>0</v>
+      <c r="E14" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -9695,15 +9695,15 @@
       <c r="D15" s="8" t="n">
         <v>5112</v>
       </c>
-      <c r="E15" s="6" t="n">
-        <v>0</v>
+      <c r="E15" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -9726,15 +9726,15 @@
       <c r="D16" s="8" t="n">
         <v>5112</v>
       </c>
-      <c r="E16" s="6" t="n">
-        <v>0</v>
+      <c r="E16" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -9788,15 +9788,15 @@
       <c r="D18" s="8" t="n">
         <v>5112</v>
       </c>
-      <c r="E18" s="6" t="n">
-        <v>0</v>
+      <c r="E18" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -9912,15 +9912,15 @@
       <c r="D22" s="8" t="n">
         <v>5112</v>
       </c>
-      <c r="E22" s="6" t="n">
-        <v>0</v>
+      <c r="E22" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -9943,15 +9943,15 @@
       <c r="D23" s="8" t="n">
         <v>5112</v>
       </c>
-      <c r="E23" s="6" t="n">
-        <v>0</v>
+      <c r="E23" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>
@@ -9974,15 +9974,15 @@
       <c r="D24" s="8" t="n">
         <v>5112</v>
       </c>
-      <c r="E24" s="6" t="n">
-        <v>0</v>
+      <c r="E24" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>✗ Lückenhaft</t>
+          <t>✓ OK</t>
         </is>
       </c>
     </row>

</xml_diff>